<commit_message>
feat: enhance export functionality and update approval logic in Compressor and WaterSoftener controllers
</commit_message>
<xml_diff>
--- a/public/assets/templates/operasional/compressor.xlsx
+++ b/public/assets/templates/operasional/compressor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\operasional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CB06BB-E763-4517-BAE5-1B1FDE6C133B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E9B9BC5-4D2C-4993-8022-880B5AB36A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{99C3DBBC-300A-4B82-A6E7-8870F6465435}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>ENGINEERING UTILITY</t>
   </si>
@@ -104,15 +104,6 @@
     <t>Disetujui Oleh</t>
   </si>
   <si>
-    <t>Operator Utility</t>
-  </si>
-  <si>
-    <t>Staff Engineering Utility</t>
-  </si>
-  <si>
-    <t>SPV Engineering Utility</t>
-  </si>
-  <si>
     <t>FRM/EUT/01/004/002-04</t>
   </si>
 </sst>
@@ -123,12 +114,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -164,6 +162,14 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -694,278 +700,301 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1334,201 +1363,201 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BE073F6-5C4D-45E5-ABA4-F18B11E1D35C}">
-  <dimension ref="A1:AC55"/>
+  <dimension ref="A1:AC56"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:29" ht="20">
-      <c r="A1" s="67"/>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="70" t="s">
+      <c r="A1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="71"/>
-      <c r="M1" s="71"/>
-      <c r="N1" s="71"/>
-      <c r="O1" s="71"/>
-      <c r="P1" s="71"/>
-      <c r="Q1" s="71"/>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71"/>
-      <c r="T1" s="71"/>
-      <c r="U1" s="71"/>
-      <c r="V1" s="71"/>
-      <c r="W1" s="71"/>
-      <c r="X1" s="71"/>
-      <c r="Y1" s="71"/>
-      <c r="Z1" s="72" t="s">
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="AA1" s="72"/>
-      <c r="AB1" s="73"/>
-      <c r="AC1" s="74"/>
+      <c r="AA1" s="28"/>
+      <c r="AB1" s="29"/>
+      <c r="AC1" s="30"/>
     </row>
     <row r="2" spans="1:29" ht="17.5">
-      <c r="A2" s="53"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="78" t="s">
+      <c r="A2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="79"/>
-      <c r="M2" s="79"/>
-      <c r="N2" s="79"/>
-      <c r="O2" s="79"/>
-      <c r="P2" s="79"/>
-      <c r="Q2" s="79"/>
-      <c r="R2" s="79"/>
-      <c r="S2" s="79"/>
-      <c r="T2" s="79"/>
-      <c r="U2" s="79"/>
-      <c r="V2" s="79"/>
-      <c r="W2" s="79"/>
-      <c r="X2" s="79"/>
-      <c r="Y2" s="79"/>
-      <c r="Z2" s="75"/>
-      <c r="AA2" s="75"/>
-      <c r="AB2" s="76"/>
-      <c r="AC2" s="77"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="35"/>
+      <c r="W2" s="35"/>
+      <c r="X2" s="35"/>
+      <c r="Y2" s="35"/>
+      <c r="Z2" s="31"/>
+      <c r="AA2" s="31"/>
+      <c r="AB2" s="32"/>
+      <c r="AC2" s="33"/>
     </row>
     <row r="3" spans="1:29" ht="15.5">
-      <c r="A3" s="45"/>
-      <c r="B3" s="80"/>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-      <c r="K3" s="80"/>
-      <c r="L3" s="80"/>
-      <c r="M3" s="80"/>
-      <c r="N3" s="80"/>
-      <c r="O3" s="80"/>
-      <c r="P3" s="80"/>
-      <c r="Q3" s="80"/>
-      <c r="R3" s="80"/>
-      <c r="S3" s="80"/>
-      <c r="T3" s="80"/>
-      <c r="U3" s="80"/>
-      <c r="V3" s="80"/>
-      <c r="W3" s="80"/>
-      <c r="X3" s="80"/>
-      <c r="Y3" s="80"/>
-      <c r="Z3" s="80"/>
-      <c r="AA3" s="80"/>
-      <c r="AB3" s="80"/>
-      <c r="AC3" s="81"/>
+      <c r="A3" s="36"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
+      <c r="I3" s="37"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="37"/>
+      <c r="L3" s="37"/>
+      <c r="M3" s="37"/>
+      <c r="N3" s="37"/>
+      <c r="O3" s="37"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="37"/>
+      <c r="R3" s="37"/>
+      <c r="S3" s="37"/>
+      <c r="T3" s="37"/>
+      <c r="U3" s="37"/>
+      <c r="V3" s="37"/>
+      <c r="W3" s="37"/>
+      <c r="X3" s="37"/>
+      <c r="Y3" s="37"/>
+      <c r="Z3" s="37"/>
+      <c r="AA3" s="37"/>
+      <c r="AB3" s="37"/>
+      <c r="AC3" s="38"/>
     </row>
     <row r="4" spans="1:29" ht="15.5">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="47"/>
-      <c r="E4" s="47"/>
-      <c r="F4" s="61"/>
-      <c r="G4" s="63" t="s">
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="56" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="64" t="s">
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="46" t="s">
+      <c r="K4" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="47"/>
-      <c r="M4" s="47"/>
-      <c r="N4" s="47"/>
-      <c r="O4" s="46" t="s">
+      <c r="L4" s="40"/>
+      <c r="M4" s="40"/>
+      <c r="N4" s="40"/>
+      <c r="O4" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="P4" s="47"/>
-      <c r="Q4" s="47"/>
-      <c r="R4" s="47"/>
-      <c r="S4" s="50" t="s">
+      <c r="P4" s="40"/>
+      <c r="Q4" s="40"/>
+      <c r="R4" s="40"/>
+      <c r="S4" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="51"/>
-      <c r="U4" s="51"/>
-      <c r="V4" s="52"/>
-      <c r="W4" s="41" t="s">
+      <c r="T4" s="44"/>
+      <c r="U4" s="44"/>
+      <c r="V4" s="45"/>
+      <c r="W4" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="X4" s="41" t="s">
+      <c r="X4" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="Y4" s="41" t="s">
+      <c r="Y4" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="Z4" s="42"/>
-      <c r="AA4" s="41" t="s">
+      <c r="Z4" s="53"/>
+      <c r="AA4" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="AB4" s="43"/>
-      <c r="AC4" s="44"/>
+      <c r="AB4" s="60"/>
+      <c r="AC4" s="61"/>
     </row>
     <row r="5" spans="1:29">
-      <c r="A5" s="42"/>
-      <c r="B5" s="42"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
-      <c r="J5" s="65"/>
-      <c r="K5" s="48"/>
-      <c r="L5" s="49"/>
-      <c r="M5" s="49"/>
-      <c r="N5" s="49"/>
-      <c r="O5" s="48"/>
-      <c r="P5" s="49"/>
-      <c r="Q5" s="49"/>
-      <c r="R5" s="49"/>
-      <c r="S5" s="53"/>
-      <c r="T5" s="54"/>
-      <c r="U5" s="54"/>
-      <c r="V5" s="55"/>
-      <c r="W5" s="41"/>
-      <c r="X5" s="42"/>
-      <c r="Y5" s="42" t="s">
+      <c r="A5" s="53"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="58"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="42"/>
+      <c r="M5" s="42"/>
+      <c r="N5" s="42"/>
+      <c r="O5" s="41"/>
+      <c r="P5" s="42"/>
+      <c r="Q5" s="42"/>
+      <c r="R5" s="42"/>
+      <c r="S5" s="23"/>
+      <c r="T5" s="24"/>
+      <c r="U5" s="24"/>
+      <c r="V5" s="25"/>
+      <c r="W5" s="47"/>
+      <c r="X5" s="53"/>
+      <c r="Y5" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="Z5" s="42" t="s">
+      <c r="Z5" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="AA5" s="42"/>
-      <c r="AB5" s="45"/>
-      <c r="AC5" s="44"/>
+      <c r="AA5" s="53"/>
+      <c r="AB5" s="36"/>
+      <c r="AC5" s="61"/>
     </row>
     <row r="6" spans="1:29" ht="15.5">
-      <c r="A6" s="42"/>
-      <c r="B6" s="42"/>
+      <c r="A6" s="53"/>
+      <c r="B6" s="53"/>
       <c r="C6" s="1">
         <v>1</v>
       </c>
@@ -1550,7 +1579,7 @@
       <c r="I6" s="4">
         <v>4</v>
       </c>
-      <c r="J6" s="66"/>
+      <c r="J6" s="59"/>
       <c r="K6" s="1">
         <v>1</v>
       </c>
@@ -1587,10 +1616,10 @@
       <c r="V6" s="1">
         <v>4</v>
       </c>
-      <c r="W6" s="41"/>
-      <c r="X6" s="42"/>
-      <c r="Y6" s="42"/>
-      <c r="Z6" s="42"/>
+      <c r="W6" s="47"/>
+      <c r="X6" s="53"/>
+      <c r="Y6" s="53"/>
+      <c r="Z6" s="53"/>
       <c r="AA6" s="1" t="s">
         <v>17</v>
       </c>
@@ -1602,7 +1631,7 @@
       </c>
     </row>
     <row r="7" spans="1:29" ht="16" thickBot="1">
-      <c r="A7" s="56"/>
+      <c r="A7" s="48"/>
       <c r="B7" s="5">
         <v>8</v>
       </c>
@@ -1635,7 +1664,7 @@
       <c r="AC7" s="8"/>
     </row>
     <row r="8" spans="1:29" ht="16" thickBot="1">
-      <c r="A8" s="57"/>
+      <c r="A8" s="49"/>
       <c r="B8" s="5">
         <v>12</v>
       </c>
@@ -1668,7 +1697,7 @@
       <c r="AC8" s="8"/>
     </row>
     <row r="9" spans="1:29" ht="16" thickBot="1">
-      <c r="A9" s="57"/>
+      <c r="A9" s="49"/>
       <c r="B9" s="5">
         <v>16</v>
       </c>
@@ -1701,7 +1730,7 @@
       <c r="AC9" s="8"/>
     </row>
     <row r="10" spans="1:29" ht="16" thickBot="1">
-      <c r="A10" s="57"/>
+      <c r="A10" s="49"/>
       <c r="B10" s="5">
         <v>20</v>
       </c>
@@ -1734,7 +1763,7 @@
       <c r="AC10" s="8"/>
     </row>
     <row r="11" spans="1:29" ht="16" thickBot="1">
-      <c r="A11" s="57"/>
+      <c r="A11" s="49"/>
       <c r="B11" s="5">
         <v>0</v>
       </c>
@@ -1767,7 +1796,7 @@
       <c r="AC11" s="8"/>
     </row>
     <row r="12" spans="1:29" ht="16" thickBot="1">
-      <c r="A12" s="57"/>
+      <c r="A12" s="49"/>
       <c r="B12" s="9">
         <v>4</v>
       </c>
@@ -1800,7 +1829,7 @@
       <c r="AC12" s="12"/>
     </row>
     <row r="13" spans="1:29" ht="16" thickBot="1">
-      <c r="A13" s="57"/>
+      <c r="A13" s="49"/>
       <c r="B13" s="5">
         <v>8</v>
       </c>
@@ -1833,7 +1862,7 @@
       <c r="AC13" s="15"/>
     </row>
     <row r="14" spans="1:29" ht="16" thickBot="1">
-      <c r="A14" s="57"/>
+      <c r="A14" s="49"/>
       <c r="B14" s="5">
         <v>12</v>
       </c>
@@ -1866,7 +1895,7 @@
       <c r="AC14" s="8"/>
     </row>
     <row r="15" spans="1:29" ht="16" thickBot="1">
-      <c r="A15" s="57"/>
+      <c r="A15" s="49"/>
       <c r="B15" s="5">
         <v>16</v>
       </c>
@@ -1899,7 +1928,7 @@
       <c r="AC15" s="8"/>
     </row>
     <row r="16" spans="1:29" ht="16" thickBot="1">
-      <c r="A16" s="57"/>
+      <c r="A16" s="49"/>
       <c r="B16" s="5">
         <v>20</v>
       </c>
@@ -1932,7 +1961,7 @@
       <c r="AC16" s="8"/>
     </row>
     <row r="17" spans="1:29" ht="16" thickBot="1">
-      <c r="A17" s="57"/>
+      <c r="A17" s="49"/>
       <c r="B17" s="5">
         <v>0</v>
       </c>
@@ -1965,7 +1994,7 @@
       <c r="AC17" s="8"/>
     </row>
     <row r="18" spans="1:29" ht="16" thickBot="1">
-      <c r="A18" s="57"/>
+      <c r="A18" s="49"/>
       <c r="B18" s="9">
         <v>4</v>
       </c>
@@ -1998,7 +2027,7 @@
       <c r="AC18" s="12"/>
     </row>
     <row r="19" spans="1:29" ht="16" thickBot="1">
-      <c r="A19" s="57"/>
+      <c r="A19" s="49"/>
       <c r="B19" s="5">
         <v>8</v>
       </c>
@@ -2031,7 +2060,7 @@
       <c r="AC19" s="15"/>
     </row>
     <row r="20" spans="1:29" ht="16" thickBot="1">
-      <c r="A20" s="57"/>
+      <c r="A20" s="49"/>
       <c r="B20" s="5">
         <v>12</v>
       </c>
@@ -2064,7 +2093,7 @@
       <c r="AC20" s="8"/>
     </row>
     <row r="21" spans="1:29" ht="16" thickBot="1">
-      <c r="A21" s="57"/>
+      <c r="A21" s="49"/>
       <c r="B21" s="5">
         <v>16</v>
       </c>
@@ -2097,7 +2126,7 @@
       <c r="AC21" s="8"/>
     </row>
     <row r="22" spans="1:29" ht="16" thickBot="1">
-      <c r="A22" s="57"/>
+      <c r="A22" s="49"/>
       <c r="B22" s="5">
         <v>20</v>
       </c>
@@ -2130,7 +2159,7 @@
       <c r="AC22" s="8"/>
     </row>
     <row r="23" spans="1:29" ht="16" thickBot="1">
-      <c r="A23" s="57"/>
+      <c r="A23" s="49"/>
       <c r="B23" s="5">
         <v>0</v>
       </c>
@@ -2163,7 +2192,7 @@
       <c r="AC23" s="8"/>
     </row>
     <row r="24" spans="1:29" ht="16" thickBot="1">
-      <c r="A24" s="57"/>
+      <c r="A24" s="49"/>
       <c r="B24" s="9">
         <v>4</v>
       </c>
@@ -2196,7 +2225,7 @@
       <c r="AC24" s="12"/>
     </row>
     <row r="25" spans="1:29" ht="16" thickBot="1">
-      <c r="A25" s="57"/>
+      <c r="A25" s="49"/>
       <c r="B25" s="5">
         <v>8</v>
       </c>
@@ -2229,7 +2258,7 @@
       <c r="AC25" s="15"/>
     </row>
     <row r="26" spans="1:29" ht="16" thickBot="1">
-      <c r="A26" s="57"/>
+      <c r="A26" s="49"/>
       <c r="B26" s="5">
         <v>12</v>
       </c>
@@ -2262,7 +2291,7 @@
       <c r="AC26" s="8"/>
     </row>
     <row r="27" spans="1:29" ht="16" thickBot="1">
-      <c r="A27" s="57"/>
+      <c r="A27" s="49"/>
       <c r="B27" s="5">
         <v>16</v>
       </c>
@@ -2295,7 +2324,7 @@
       <c r="AC27" s="8"/>
     </row>
     <row r="28" spans="1:29" ht="16" thickBot="1">
-      <c r="A28" s="57"/>
+      <c r="A28" s="49"/>
       <c r="B28" s="5">
         <v>20</v>
       </c>
@@ -2328,7 +2357,7 @@
       <c r="AC28" s="8"/>
     </row>
     <row r="29" spans="1:29" ht="16" thickBot="1">
-      <c r="A29" s="57"/>
+      <c r="A29" s="49"/>
       <c r="B29" s="5">
         <v>0</v>
       </c>
@@ -2361,7 +2390,7 @@
       <c r="AC29" s="8"/>
     </row>
     <row r="30" spans="1:29" ht="16" thickBot="1">
-      <c r="A30" s="57"/>
+      <c r="A30" s="49"/>
       <c r="B30" s="9">
         <v>4</v>
       </c>
@@ -2394,7 +2423,7 @@
       <c r="AC30" s="12"/>
     </row>
     <row r="31" spans="1:29" ht="15.5">
-      <c r="A31" s="58"/>
+      <c r="A31" s="50"/>
       <c r="B31" s="5">
         <v>8</v>
       </c>
@@ -2427,7 +2456,7 @@
       <c r="AC31" s="15"/>
     </row>
     <row r="32" spans="1:29" ht="15.5">
-      <c r="A32" s="59"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="5">
         <v>12</v>
       </c>
@@ -2460,7 +2489,7 @@
       <c r="AC32" s="8"/>
     </row>
     <row r="33" spans="1:29" ht="15.5">
-      <c r="A33" s="59"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="5">
         <v>16</v>
       </c>
@@ -2493,7 +2522,7 @@
       <c r="AC33" s="8"/>
     </row>
     <row r="34" spans="1:29" ht="15.5">
-      <c r="A34" s="59"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="5">
         <v>20</v>
       </c>
@@ -2526,7 +2555,7 @@
       <c r="AC34" s="8"/>
     </row>
     <row r="35" spans="1:29" ht="15.5">
-      <c r="A35" s="59"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="5">
         <v>0</v>
       </c>
@@ -2559,7 +2588,7 @@
       <c r="AC35" s="8"/>
     </row>
     <row r="36" spans="1:29" ht="16" thickBot="1">
-      <c r="A36" s="60"/>
+      <c r="A36" s="52"/>
       <c r="B36" s="9">
         <v>4</v>
       </c>
@@ -2592,7 +2621,7 @@
       <c r="AC36" s="12"/>
     </row>
     <row r="37" spans="1:29" ht="16" thickBot="1">
-      <c r="A37" s="26"/>
+      <c r="A37" s="46"/>
       <c r="B37" s="5">
         <v>8</v>
       </c>
@@ -2625,7 +2654,7 @@
       <c r="AC37" s="15"/>
     </row>
     <row r="38" spans="1:29" ht="16" thickBot="1">
-      <c r="A38" s="26"/>
+      <c r="A38" s="46"/>
       <c r="B38" s="5">
         <v>12</v>
       </c>
@@ -2658,7 +2687,7 @@
       <c r="AC38" s="8"/>
     </row>
     <row r="39" spans="1:29" ht="16" thickBot="1">
-      <c r="A39" s="26"/>
+      <c r="A39" s="46"/>
       <c r="B39" s="5">
         <v>16</v>
       </c>
@@ -2691,7 +2720,7 @@
       <c r="AC39" s="8"/>
     </row>
     <row r="40" spans="1:29" ht="16" thickBot="1">
-      <c r="A40" s="26"/>
+      <c r="A40" s="46"/>
       <c r="B40" s="5">
         <v>20</v>
       </c>
@@ -2724,7 +2753,7 @@
       <c r="AC40" s="8"/>
     </row>
     <row r="41" spans="1:29" ht="16" thickBot="1">
-      <c r="A41" s="26"/>
+      <c r="A41" s="46"/>
       <c r="B41" s="5">
         <v>0</v>
       </c>
@@ -2757,7 +2786,7 @@
       <c r="AC41" s="8"/>
     </row>
     <row r="42" spans="1:29" ht="16" thickBot="1">
-      <c r="A42" s="26"/>
+      <c r="A42" s="46"/>
       <c r="B42" s="9">
         <v>4</v>
       </c>
@@ -2790,7 +2819,7 @@
       <c r="AC42" s="12"/>
     </row>
     <row r="43" spans="1:29" ht="16" thickBot="1">
-      <c r="A43" s="26"/>
+      <c r="A43" s="46"/>
       <c r="B43" s="5">
         <v>8</v>
       </c>
@@ -2823,7 +2852,7 @@
       <c r="AC43" s="15"/>
     </row>
     <row r="44" spans="1:29" ht="16" thickBot="1">
-      <c r="A44" s="26"/>
+      <c r="A44" s="46"/>
       <c r="B44" s="5">
         <v>12</v>
       </c>
@@ -2856,7 +2885,7 @@
       <c r="AC44" s="8"/>
     </row>
     <row r="45" spans="1:29" ht="16" thickBot="1">
-      <c r="A45" s="26"/>
+      <c r="A45" s="46"/>
       <c r="B45" s="5">
         <v>16</v>
       </c>
@@ -2889,7 +2918,7 @@
       <c r="AC45" s="8"/>
     </row>
     <row r="46" spans="1:29" ht="16" thickBot="1">
-      <c r="A46" s="26"/>
+      <c r="A46" s="46"/>
       <c r="B46" s="5">
         <v>20</v>
       </c>
@@ -2922,7 +2951,7 @@
       <c r="AC46" s="8"/>
     </row>
     <row r="47" spans="1:29" ht="16" thickBot="1">
-      <c r="A47" s="26"/>
+      <c r="A47" s="46"/>
       <c r="B47" s="5">
         <v>0</v>
       </c>
@@ -2955,7 +2984,7 @@
       <c r="AC47" s="8"/>
     </row>
     <row r="48" spans="1:29" ht="16" thickBot="1">
-      <c r="A48" s="27"/>
+      <c r="A48" s="62"/>
       <c r="B48" s="9">
         <v>4</v>
       </c>
@@ -2988,245 +3017,284 @@
       <c r="AC48" s="8"/>
     </row>
     <row r="49" spans="1:29" ht="15">
-      <c r="A49" s="28" t="s">
+      <c r="A49" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="B49" s="29"/>
-      <c r="C49" s="29"/>
-      <c r="D49" s="29"/>
-      <c r="E49" s="29"/>
-      <c r="F49" s="29"/>
-      <c r="G49" s="29"/>
-      <c r="H49" s="29"/>
-      <c r="I49" s="29"/>
-      <c r="J49" s="29"/>
-      <c r="K49" s="29"/>
-      <c r="L49" s="29"/>
-      <c r="M49" s="29"/>
-      <c r="N49" s="29"/>
-      <c r="O49" s="29"/>
-      <c r="P49" s="29"/>
-      <c r="Q49" s="29"/>
-      <c r="R49" s="29"/>
-      <c r="S49" s="29"/>
-      <c r="T49" s="29"/>
-      <c r="U49" s="29"/>
-      <c r="V49" s="29"/>
-      <c r="W49" s="29"/>
-      <c r="X49" s="29"/>
-      <c r="Y49" s="29"/>
-      <c r="Z49" s="29"/>
-      <c r="AA49" s="29"/>
-      <c r="AB49" s="30"/>
-      <c r="AC49" s="31"/>
+      <c r="B49" s="64"/>
+      <c r="C49" s="64"/>
+      <c r="D49" s="64"/>
+      <c r="E49" s="64"/>
+      <c r="F49" s="64"/>
+      <c r="G49" s="64"/>
+      <c r="H49" s="64"/>
+      <c r="I49" s="64"/>
+      <c r="J49" s="64"/>
+      <c r="K49" s="64"/>
+      <c r="L49" s="64"/>
+      <c r="M49" s="64"/>
+      <c r="N49" s="64"/>
+      <c r="O49" s="64"/>
+      <c r="P49" s="64"/>
+      <c r="Q49" s="64"/>
+      <c r="R49" s="64"/>
+      <c r="S49" s="64"/>
+      <c r="T49" s="64"/>
+      <c r="U49" s="64"/>
+      <c r="V49" s="64"/>
+      <c r="W49" s="64"/>
+      <c r="X49" s="64"/>
+      <c r="Y49" s="64"/>
+      <c r="Z49" s="64"/>
+      <c r="AA49" s="64"/>
+      <c r="AB49" s="65"/>
+      <c r="AC49" s="66"/>
     </row>
     <row r="50" spans="1:29" ht="18">
-      <c r="A50" s="32" t="s">
+      <c r="A50" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="33"/>
-      <c r="C50" s="33"/>
-      <c r="D50" s="33"/>
-      <c r="E50" s="33"/>
-      <c r="F50" s="33"/>
-      <c r="G50" s="33"/>
-      <c r="H50" s="33"/>
-      <c r="I50" s="33"/>
-      <c r="J50" s="34" t="s">
+      <c r="B50" s="68"/>
+      <c r="C50" s="68"/>
+      <c r="D50" s="68"/>
+      <c r="E50" s="68"/>
+      <c r="F50" s="68"/>
+      <c r="G50" s="68"/>
+      <c r="H50" s="68"/>
+      <c r="I50" s="68"/>
+      <c r="J50" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="K50" s="33"/>
-      <c r="L50" s="33"/>
-      <c r="M50" s="33"/>
-      <c r="N50" s="33"/>
-      <c r="O50" s="33"/>
-      <c r="P50" s="33"/>
-      <c r="Q50" s="33"/>
-      <c r="R50" s="33"/>
-      <c r="S50" s="35"/>
-      <c r="T50" s="36" t="s">
+      <c r="K50" s="68"/>
+      <c r="L50" s="68"/>
+      <c r="M50" s="68"/>
+      <c r="N50" s="68"/>
+      <c r="O50" s="68"/>
+      <c r="P50" s="68"/>
+      <c r="Q50" s="68"/>
+      <c r="R50" s="68"/>
+      <c r="S50" s="70"/>
+      <c r="T50" s="71" t="s">
         <v>23</v>
       </c>
-      <c r="U50" s="36"/>
-      <c r="V50" s="36"/>
-      <c r="W50" s="36"/>
-      <c r="X50" s="36"/>
-      <c r="Y50" s="36"/>
-      <c r="Z50" s="36"/>
-      <c r="AA50" s="36"/>
-      <c r="AB50" s="34"/>
-      <c r="AC50" s="37"/>
+      <c r="U50" s="71"/>
+      <c r="V50" s="71"/>
+      <c r="W50" s="71"/>
+      <c r="X50" s="71"/>
+      <c r="Y50" s="71"/>
+      <c r="Z50" s="71"/>
+      <c r="AA50" s="71"/>
+      <c r="AB50" s="69"/>
+      <c r="AC50" s="72"/>
     </row>
     <row r="51" spans="1:29">
-      <c r="A51" s="82"/>
-      <c r="B51" s="83"/>
-      <c r="C51" s="83"/>
-      <c r="D51" s="83"/>
-      <c r="E51" s="83"/>
-      <c r="F51" s="83"/>
-      <c r="G51" s="83"/>
-      <c r="H51" s="83"/>
-      <c r="I51" s="84"/>
-      <c r="J51" s="38"/>
-      <c r="K51" s="38"/>
-      <c r="L51" s="38"/>
-      <c r="M51" s="38"/>
-      <c r="N51" s="38"/>
-      <c r="O51" s="38"/>
-      <c r="P51" s="38"/>
-      <c r="Q51" s="38"/>
-      <c r="R51" s="38"/>
-      <c r="S51" s="38"/>
-      <c r="T51" s="38"/>
-      <c r="U51" s="38"/>
-      <c r="V51" s="38"/>
-      <c r="W51" s="38"/>
-      <c r="X51" s="38"/>
-      <c r="Y51" s="38"/>
-      <c r="Z51" s="38"/>
-      <c r="AA51" s="38"/>
-      <c r="AB51" s="39"/>
-      <c r="AC51" s="40"/>
+      <c r="A51" s="73"/>
+      <c r="B51" s="74"/>
+      <c r="C51" s="74"/>
+      <c r="D51" s="74"/>
+      <c r="E51" s="74"/>
+      <c r="F51" s="74"/>
+      <c r="G51" s="74"/>
+      <c r="H51" s="74"/>
+      <c r="I51" s="75"/>
+      <c r="J51" s="82"/>
+      <c r="K51" s="82"/>
+      <c r="L51" s="82"/>
+      <c r="M51" s="82"/>
+      <c r="N51" s="82"/>
+      <c r="O51" s="82"/>
+      <c r="P51" s="82"/>
+      <c r="Q51" s="82"/>
+      <c r="R51" s="82"/>
+      <c r="S51" s="82"/>
+      <c r="T51" s="82"/>
+      <c r="U51" s="82"/>
+      <c r="V51" s="82"/>
+      <c r="W51" s="82"/>
+      <c r="X51" s="82"/>
+      <c r="Y51" s="82"/>
+      <c r="Z51" s="82"/>
+      <c r="AA51" s="82"/>
+      <c r="AB51" s="83"/>
+      <c r="AC51" s="84"/>
     </row>
     <row r="52" spans="1:29">
-      <c r="A52" s="85"/>
-      <c r="B52" s="86"/>
-      <c r="C52" s="86"/>
-      <c r="D52" s="86"/>
-      <c r="E52" s="86"/>
-      <c r="F52" s="86"/>
-      <c r="G52" s="86"/>
-      <c r="H52" s="86"/>
-      <c r="I52" s="87"/>
-      <c r="J52" s="38"/>
-      <c r="K52" s="38"/>
-      <c r="L52" s="38"/>
-      <c r="M52" s="38"/>
-      <c r="N52" s="38"/>
-      <c r="O52" s="38"/>
-      <c r="P52" s="38"/>
-      <c r="Q52" s="38"/>
-      <c r="R52" s="38"/>
-      <c r="S52" s="38"/>
-      <c r="T52" s="38"/>
-      <c r="U52" s="38"/>
-      <c r="V52" s="38"/>
-      <c r="W52" s="38"/>
-      <c r="X52" s="38"/>
-      <c r="Y52" s="38"/>
-      <c r="Z52" s="38"/>
-      <c r="AA52" s="38"/>
-      <c r="AB52" s="39"/>
-      <c r="AC52" s="40"/>
+      <c r="A52" s="76"/>
+      <c r="B52" s="77"/>
+      <c r="C52" s="77"/>
+      <c r="D52" s="77"/>
+      <c r="E52" s="77"/>
+      <c r="F52" s="77"/>
+      <c r="G52" s="77"/>
+      <c r="H52" s="77"/>
+      <c r="I52" s="78"/>
+      <c r="J52" s="82"/>
+      <c r="K52" s="82"/>
+      <c r="L52" s="82"/>
+      <c r="M52" s="82"/>
+      <c r="N52" s="82"/>
+      <c r="O52" s="82"/>
+      <c r="P52" s="82"/>
+      <c r="Q52" s="82"/>
+      <c r="R52" s="82"/>
+      <c r="S52" s="82"/>
+      <c r="T52" s="82"/>
+      <c r="U52" s="82"/>
+      <c r="V52" s="82"/>
+      <c r="W52" s="82"/>
+      <c r="X52" s="82"/>
+      <c r="Y52" s="82"/>
+      <c r="Z52" s="82"/>
+      <c r="AA52" s="82"/>
+      <c r="AB52" s="83"/>
+      <c r="AC52" s="84"/>
     </row>
     <row r="53" spans="1:29">
-      <c r="A53" s="88"/>
-      <c r="B53" s="89"/>
-      <c r="C53" s="89"/>
-      <c r="D53" s="89"/>
-      <c r="E53" s="89"/>
-      <c r="F53" s="89"/>
-      <c r="G53" s="89"/>
-      <c r="H53" s="89"/>
-      <c r="I53" s="90"/>
-      <c r="J53" s="38"/>
-      <c r="K53" s="38"/>
-      <c r="L53" s="38"/>
-      <c r="M53" s="38"/>
-      <c r="N53" s="38"/>
-      <c r="O53" s="38"/>
-      <c r="P53" s="38"/>
-      <c r="Q53" s="38"/>
-      <c r="R53" s="38"/>
-      <c r="S53" s="38"/>
-      <c r="T53" s="38"/>
-      <c r="U53" s="38"/>
-      <c r="V53" s="38"/>
-      <c r="W53" s="38"/>
-      <c r="X53" s="38"/>
-      <c r="Y53" s="38"/>
-      <c r="Z53" s="38"/>
-      <c r="AA53" s="38"/>
-      <c r="AB53" s="39"/>
-      <c r="AC53" s="40"/>
-    </row>
-    <row r="54" spans="1:29" ht="18" thickBot="1">
-      <c r="A54" s="20" t="s">
+      <c r="A53" s="79"/>
+      <c r="B53" s="80"/>
+      <c r="C53" s="80"/>
+      <c r="D53" s="80"/>
+      <c r="E53" s="80"/>
+      <c r="F53" s="80"/>
+      <c r="G53" s="80"/>
+      <c r="H53" s="80"/>
+      <c r="I53" s="81"/>
+      <c r="J53" s="82"/>
+      <c r="K53" s="82"/>
+      <c r="L53" s="82"/>
+      <c r="M53" s="82"/>
+      <c r="N53" s="82"/>
+      <c r="O53" s="82"/>
+      <c r="P53" s="82"/>
+      <c r="Q53" s="82"/>
+      <c r="R53" s="82"/>
+      <c r="S53" s="82"/>
+      <c r="T53" s="82"/>
+      <c r="U53" s="82"/>
+      <c r="V53" s="82"/>
+      <c r="W53" s="82"/>
+      <c r="X53" s="82"/>
+      <c r="Y53" s="82"/>
+      <c r="Z53" s="82"/>
+      <c r="AA53" s="82"/>
+      <c r="AB53" s="83"/>
+      <c r="AC53" s="84"/>
+    </row>
+    <row r="54" spans="1:29" s="99" customFormat="1" ht="17.5">
+      <c r="A54" s="92"/>
+      <c r="B54" s="93"/>
+      <c r="C54" s="93"/>
+      <c r="D54" s="93"/>
+      <c r="E54" s="93"/>
+      <c r="F54" s="93"/>
+      <c r="G54" s="93"/>
+      <c r="H54" s="93"/>
+      <c r="I54" s="94"/>
+      <c r="J54" s="95"/>
+      <c r="K54" s="96"/>
+      <c r="L54" s="96"/>
+      <c r="M54" s="96"/>
+      <c r="N54" s="96"/>
+      <c r="O54" s="96"/>
+      <c r="P54" s="96"/>
+      <c r="Q54" s="96"/>
+      <c r="R54" s="96"/>
+      <c r="S54" s="97"/>
+      <c r="T54" s="95"/>
+      <c r="U54" s="96"/>
+      <c r="V54" s="96"/>
+      <c r="W54" s="96"/>
+      <c r="X54" s="96"/>
+      <c r="Y54" s="96"/>
+      <c r="Z54" s="96"/>
+      <c r="AA54" s="96"/>
+      <c r="AB54" s="96"/>
+      <c r="AC54" s="98"/>
+    </row>
+    <row r="55" spans="1:29" s="91" customFormat="1" ht="18.5" thickBot="1">
+      <c r="A55" s="85"/>
+      <c r="B55" s="86"/>
+      <c r="C55" s="86"/>
+      <c r="D55" s="86"/>
+      <c r="E55" s="86"/>
+      <c r="F55" s="86"/>
+      <c r="G55" s="86"/>
+      <c r="H55" s="86"/>
+      <c r="I55" s="87"/>
+      <c r="J55" s="88"/>
+      <c r="K55" s="88"/>
+      <c r="L55" s="88"/>
+      <c r="M55" s="88"/>
+      <c r="N55" s="88"/>
+      <c r="O55" s="88"/>
+      <c r="P55" s="88"/>
+      <c r="Q55" s="88"/>
+      <c r="R55" s="88"/>
+      <c r="S55" s="88"/>
+      <c r="T55" s="88"/>
+      <c r="U55" s="88"/>
+      <c r="V55" s="88"/>
+      <c r="W55" s="88"/>
+      <c r="X55" s="88"/>
+      <c r="Y55" s="88"/>
+      <c r="Z55" s="88"/>
+      <c r="AA55" s="88"/>
+      <c r="AB55" s="89"/>
+      <c r="AC55" s="90"/>
+    </row>
+    <row r="56" spans="1:29" ht="15.5">
+      <c r="A56" s="17"/>
+      <c r="B56" s="17"/>
+      <c r="C56" s="17"/>
+      <c r="D56" s="17"/>
+      <c r="E56" s="17"/>
+      <c r="F56" s="17"/>
+      <c r="G56" s="17"/>
+      <c r="H56" s="17"/>
+      <c r="I56" s="17"/>
+      <c r="J56" s="17"/>
+      <c r="K56" s="17"/>
+      <c r="L56" s="17"/>
+      <c r="M56" s="17"/>
+      <c r="N56" s="17"/>
+      <c r="O56" s="17"/>
+      <c r="P56" s="17"/>
+      <c r="Q56" s="17"/>
+      <c r="R56" s="17"/>
+      <c r="S56" s="17"/>
+      <c r="T56" s="17"/>
+      <c r="U56" s="17"/>
+      <c r="V56" s="17"/>
+      <c r="W56" s="17"/>
+      <c r="X56" s="17"/>
+      <c r="Y56" s="17"/>
+      <c r="Z56" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B54" s="21"/>
-      <c r="C54" s="21"/>
-      <c r="D54" s="21"/>
-      <c r="E54" s="21"/>
-      <c r="F54" s="21"/>
-      <c r="G54" s="21"/>
-      <c r="H54" s="21"/>
-      <c r="I54" s="22"/>
-      <c r="J54" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="K54" s="23"/>
-      <c r="L54" s="23"/>
-      <c r="M54" s="23"/>
-      <c r="N54" s="23"/>
-      <c r="O54" s="23"/>
-      <c r="P54" s="23"/>
-      <c r="Q54" s="23"/>
-      <c r="R54" s="23"/>
-      <c r="S54" s="23"/>
-      <c r="T54" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="U54" s="23"/>
-      <c r="V54" s="23"/>
-      <c r="W54" s="23"/>
-      <c r="X54" s="23"/>
-      <c r="Y54" s="23"/>
-      <c r="Z54" s="23"/>
-      <c r="AA54" s="23"/>
-      <c r="AB54" s="24"/>
-      <c r="AC54" s="25"/>
-    </row>
-    <row r="55" spans="1:29" ht="15.5">
-      <c r="A55" s="17"/>
-      <c r="B55" s="17"/>
-      <c r="C55" s="17"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="17"/>
-      <c r="G55" s="17"/>
-      <c r="H55" s="17"/>
-      <c r="I55" s="17"/>
-      <c r="J55" s="17"/>
-      <c r="K55" s="17"/>
-      <c r="L55" s="17"/>
-      <c r="M55" s="17"/>
-      <c r="N55" s="17"/>
-      <c r="O55" s="17"/>
-      <c r="P55" s="17"/>
-      <c r="Q55" s="17"/>
-      <c r="R55" s="17"/>
-      <c r="S55" s="17"/>
-      <c r="T55" s="17"/>
-      <c r="U55" s="17"/>
-      <c r="V55" s="17"/>
-      <c r="W55" s="17"/>
-      <c r="X55" s="17"/>
-      <c r="Y55" s="17"/>
-      <c r="Z55" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA55" s="19"/>
-      <c r="AB55" s="18"/>
-      <c r="AC55" s="19"/>
+      <c r="AA56" s="19"/>
+      <c r="AB56" s="18"/>
+      <c r="AC56" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="A1:G2"/>
-    <mergeCell ref="H1:Y1"/>
-    <mergeCell ref="Z1:AC2"/>
-    <mergeCell ref="H2:Y2"/>
-    <mergeCell ref="A3:AC3"/>
+  <mergeCells count="39">
+    <mergeCell ref="A55:I55"/>
+    <mergeCell ref="J55:S55"/>
+    <mergeCell ref="T55:AC55"/>
+    <mergeCell ref="A43:A48"/>
+    <mergeCell ref="A49:AC49"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="J50:S50"/>
+    <mergeCell ref="T50:AC50"/>
+    <mergeCell ref="A51:I53"/>
+    <mergeCell ref="J51:S53"/>
+    <mergeCell ref="T51:AC53"/>
+    <mergeCell ref="A54:I54"/>
+    <mergeCell ref="J54:S54"/>
+    <mergeCell ref="T54:AC54"/>
+    <mergeCell ref="X4:X6"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AA4:AC5"/>
+    <mergeCell ref="Y5:Y6"/>
+    <mergeCell ref="Z5:Z6"/>
     <mergeCell ref="K4:N5"/>
     <mergeCell ref="O4:R5"/>
     <mergeCell ref="S4:V5"/>
@@ -3242,22 +3310,11 @@
     <mergeCell ref="C4:F5"/>
     <mergeCell ref="G4:I5"/>
     <mergeCell ref="J4:J6"/>
-    <mergeCell ref="X4:X6"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AA4:AC5"/>
-    <mergeCell ref="Y5:Y6"/>
-    <mergeCell ref="Z5:Z6"/>
-    <mergeCell ref="A54:I54"/>
-    <mergeCell ref="J54:S54"/>
-    <mergeCell ref="T54:AC54"/>
-    <mergeCell ref="A43:A48"/>
-    <mergeCell ref="A49:AC49"/>
-    <mergeCell ref="A50:I50"/>
-    <mergeCell ref="J50:S50"/>
-    <mergeCell ref="T50:AC50"/>
-    <mergeCell ref="A51:I53"/>
-    <mergeCell ref="J51:S53"/>
-    <mergeCell ref="T51:AC53"/>
+    <mergeCell ref="A1:G2"/>
+    <mergeCell ref="H1:Y1"/>
+    <mergeCell ref="Z1:AC2"/>
+    <mergeCell ref="H2:Y2"/>
+    <mergeCell ref="A3:AC3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>